<commit_message>
Write down how branches and layouts pair up
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/V2.xlsx
+++ b/V2.xlsx
@@ -8,14 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matiastorrilla/projects/TV-Strats/Node/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB396CE-2467-5043-9AAD-D7897988F1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADC6DB0-6E49-0C40-A8CB-6726B091D640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{CB8A66BD-079F-D040-AABD-E821572FC271}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{CB8A66BD-079F-D040-AABD-E821572FC271}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Business Objects" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$14</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,14 +40,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="69">
   <si>
     <t>Cluster H4</t>
   </si>
   <si>
-    <t>Investor Latent Orders</t>
-  </si>
-  <si>
     <t>Trend Following Strategy</t>
   </si>
   <si>
@@ -109,9 +111,6 @@
     <t>Trend Object (Previous day collapses),ID Trend Collapses, sin opposite (LONG)</t>
   </si>
   <si>
-    <t>Feriado</t>
-  </si>
-  <si>
     <t>Cluster H4 (Swing Trend)</t>
   </si>
   <si>
@@ -146,13 +145,115 @@
   </si>
   <si>
     <t>Cluster H4 (previous day) (con imbalance)</t>
+  </si>
+  <si>
+    <t>Actual day highs liquidated.</t>
+  </si>
+  <si>
+    <t>Sin opposite Object (SHORT)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Holliday</t>
+  </si>
+  <si>
+    <t>No Position</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Reversal Strategy/Trend Following Strategy</t>
+  </si>
+  <si>
+    <t>el setup se armo antes</t>
+  </si>
+  <si>
+    <t>Positional</t>
+  </si>
+  <si>
+    <t>Investor</t>
+  </si>
+  <si>
+    <t>Swing</t>
+  </si>
+  <si>
+    <t>Latent objects</t>
+  </si>
+  <si>
+    <t>Break and Retest</t>
+  </si>
+  <si>
+    <t>Investor, Positional, Swing</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>3 a 7 días</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>Classes</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Timeframe</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>3 o mas</t>
+  </si>
+  <si>
+    <t>H4</t>
+  </si>
+  <si>
+    <t>Swing, Momentum</t>
+  </si>
+  <si>
+    <t>Sub-class</t>
+  </si>
+  <si>
+    <t>Imbalance, Balance</t>
+  </si>
+  <si>
+    <t>Events</t>
+  </si>
+  <si>
+    <t>Price achieved</t>
+  </si>
+  <si>
+    <t>Actual day high achieved, Actual day low achieved, NY Low achieved, NY High Achieved</t>
+  </si>
+  <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>No opposite object</t>
+  </si>
+  <si>
+    <t>LONG, SHORT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -168,16 +269,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -185,15 +300,90 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -509,252 +699,810 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D022E1A0-C7E2-E240-878A-1BF7152AE85E}">
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L70"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="66.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="4" width="40" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="66.33203125" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="13" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="0" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <f>A2+1</f>
+        <v>46205</v>
+      </c>
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>46204</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <f>A3+1</f>
+        <v>46206</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>46205</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>46206</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <f>A4+1</f>
+        <v>46207</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="4">
+        <f>A2+6</f>
+        <v>46210</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>46207</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>46210</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="G6" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <f>A6+1</f>
+        <v>46211</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>46211</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>27</v>
+      <c r="G7" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
+      <c r="A8" s="3">
+        <f>A7+1</f>
         <v>46212</v>
       </c>
       <c r="C8" t="s">
         <v>0</v>
       </c>
       <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" t="s">
+      <c r="G8" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <f>A8+1</f>
+        <v>46213</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
         <v>29</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F9" t="s">
         <v>30</v>
       </c>
-      <c r="G8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>46213</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <f>A9+1</f>
+        <v>46214</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
         <v>31</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="4">
+        <f>A6+7</f>
+        <v>46217</v>
+      </c>
+      <c r="D11" t="s">
         <v>32</v>
       </c>
-      <c r="G9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>46214</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <f>A11+1</f>
+        <v>46218</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
         <v>33</v>
       </c>
-      <c r="F10" t="s">
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" t="s">
         <v>30</v>
       </c>
-      <c r="G10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>46215</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="G12" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <f t="shared" ref="A13:A20" si="0">A12+1</f>
+        <v>46219</v>
+      </c>
+      <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="E11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="F13" t="s">
         <v>30</v>
       </c>
-      <c r="G11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>46218</v>
-      </c>
-      <c r="C12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="G13" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <f t="shared" si="0"/>
+        <v>46220</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
         <v>35</v>
       </c>
-      <c r="E12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F12" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>46219</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="E14" t="s">
         <v>36</v>
       </c>
-      <c r="F13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" t="s">
-        <v>10</v>
-      </c>
+      <c r="F14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <f t="shared" si="0"/>
+        <v>46221</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="4">
+        <f>A11+7</f>
+        <v>46224</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <f>A16+1</f>
+        <v>46225</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <f t="shared" si="0"/>
+        <v>46226</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <f t="shared" si="0"/>
+        <v>46227</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <f t="shared" si="0"/>
+        <v>46228</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="4">
+        <f>A16+7</f>
+        <v>46231</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <f>A21+1</f>
+        <v>46232</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <f t="shared" ref="A23:A30" si="1">A22+1</f>
+        <v>46233</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <f t="shared" si="1"/>
+        <v>46234</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <f t="shared" si="1"/>
+        <v>46235</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="4">
+        <f>A21+7</f>
+        <v>46238</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <f>A26+1</f>
+        <v>46239</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <f t="shared" si="1"/>
+        <v>46240</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <f t="shared" si="1"/>
+        <v>46241</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <f t="shared" si="1"/>
+        <v>46242</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="4">
+        <f>A26+7</f>
+        <v>46245</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <f>A31+1</f>
+        <v>46246</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <f t="shared" ref="A33:A40" si="2">A32+1</f>
+        <v>46247</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <f t="shared" si="2"/>
+        <v>46248</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <f t="shared" si="2"/>
+        <v>46249</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="4">
+        <f>A31+7</f>
+        <v>46252</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <f>A36+1</f>
+        <v>46253</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <f t="shared" si="2"/>
+        <v>46254</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <f t="shared" si="2"/>
+        <v>46255</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <f t="shared" si="2"/>
+        <v>46256</v>
+      </c>
+      <c r="B40" t="s">
+        <v>45</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A41" s="4">
+        <f>A36+7</f>
+        <v>46259</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <f>A41+1</f>
+        <v>46260</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <f t="shared" ref="A43:A50" si="3">A42+1</f>
+        <v>46261</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <f t="shared" si="3"/>
+        <v>46262</v>
+      </c>
+      <c r="B44" t="s">
+        <v>45</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <f t="shared" si="3"/>
+        <v>46263</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A46" s="4">
+        <f>A41+7</f>
+        <v>46266</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <f>A46+1</f>
+        <v>46267</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <f t="shared" si="3"/>
+        <v>46268</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <f t="shared" si="3"/>
+        <v>46269</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <f t="shared" si="3"/>
+        <v>46270</v>
+      </c>
+      <c r="B50" t="s">
+        <v>45</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="4">
+        <f>A46+7</f>
+        <v>46273</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <f>A51+1</f>
+        <v>46274</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <f t="shared" ref="A53:A60" si="4">A52+1</f>
+        <v>46275</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <f t="shared" si="4"/>
+        <v>46276</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="3">
+        <f t="shared" si="4"/>
+        <v>46277</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="4">
+        <f>A51+7</f>
+        <v>46280</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <f>A56+1</f>
+        <v>46281</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <f t="shared" si="4"/>
+        <v>46282</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <f t="shared" si="4"/>
+        <v>46283</v>
+      </c>
+      <c r="B59" t="s">
+        <v>45</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <f t="shared" si="4"/>
+        <v>46284</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="4">
+        <f>A56+7</f>
+        <v>46287</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
+        <f>A61+1</f>
+        <v>46288</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
+        <f>A62+1</f>
+        <v>46289</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
+        <f>A63+1</f>
+        <v>46290</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
+        <f>A64+1</f>
+        <v>46291</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" s="4">
+        <f>A61+7</f>
+        <v>46294</v>
+      </c>
+      <c r="B66" t="s">
+        <v>45</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
+        <f>A66+1</f>
+        <v>46295</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" s="6"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="6"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K14" xr:uid="{D022E1A0-C7E2-E240-878A-1BF7152AE85E}"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{50C65B1A-278E-FD42-B9F8-5996EAA74982}">
+      <formula1>"Trend Following Strategy,Reversal Strategy,Reversal Strategy/Trend Following Strategy,No Position,Holliday"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{48DF23FB-E18A-0D4D-8AC9-883BA511D644}">
+      <formula1>"Swing,Positional,Investor"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" xr:uid="{FC8CA7E0-C302-E449-AFFF-278F33562EA1}"/>
     <hyperlink ref="I3" r:id="rId2" xr:uid="{2ED19733-FC11-0241-85C3-CCF7464D5C3F}"/>
@@ -767,4 +1515,154 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71875A64-6CB0-9845-AE46-9C3DF5BAC46F}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="74.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C1" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B11" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B17" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B20" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>